<commit_message>
[FieldObject Data] 데이터 추가 - 토마토 주스
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/FieldObject.xlsx
+++ b/JsonConverter/ExcelFiles/FieldObject.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.12458"/>
+  <x:fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.12581"/>
   <x:workbookPr date1904="0" showBorderUnselectedTables="1" filterPrivacy="0" promptedSolutions="0" showInkAnnotation="1" backupFile="0" saveExternalLinkValues="1" codeName="ThisWorkbook" hidePivotFieldList="0" allowRefreshQuery="0" publishItems="0" checkCompatibility="0" autoCompressPictures="1" refreshAllConnections="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BootCamp\2D_Evaulation\JsonConverter\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BootCamp\2DProject\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="18852" windowHeight="6744"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="30468" windowHeight="12840"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId4"/>
@@ -19,105 +19,117 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
+  <x:si>
+    <x:t>10,1000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Harvest</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10,100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int[]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>드랍된 금화</x:t>
+  </x:si>
+  <x:si>
+    <x:t>감자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>옥수수</x:t>
+  </x:si>
+  <x:si>
+    <x:t>금화</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_TomatoJuice_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토마토 주스</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Corn_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DropItem</x:t>
+  </x:si>
+  <x:si>
+    <x:t>필드 채집용 옥수수</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PrefabPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Gold_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>필드 채집용 감자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>harv_corn_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DropCountRange</x:t>
+  </x:si>
+  <x:si>
+    <x:t>harv_potato_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>우선 프리팹으로 구현하자!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DropItemDataId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Potato_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dropItem_gold_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몬스터 설명 (도감용)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FieldObjectType</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DPrefab/Harvest_Potato</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DPrefab/Harvest_Corn</x:t>
+  </x:si>
   <x:si>
     <x:t>2DPrefab/DropItem_Gold</x:t>
   </x:si>
   <x:si>
-    <x:t>2DPrefab/Harvest_Potato</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DPrefab/Harvest_Corn</x:t>
-  </x:si>
-  <x:si>
-    <x:t>금화</x:t>
-  </x:si>
-  <x:si>
-    <x:t>감자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>옥수수</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10,1000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Harvest</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int[]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>드랍된 금화</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10,100</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dropItem_gold_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FieldObjectType</x:t>
-  </x:si>
-  <x:si>
-    <x:t>harv_potato_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Potato_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몬스터 설명 (도감용)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DropCountRange</x:t>
-  </x:si>
-  <x:si>
-    <x:t>우선 프리팹으로 구현하자!</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DropItemDataId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>필드 채집용 옥수수</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Corn_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>harv_corn_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PrefabPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DropItem</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Gold_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>필드 채집용 감자</x:t>
+    <x:t>2DPrefab/DropItem_TomatoJuice</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dropItem_tomatoJuice_1</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -977,11 +989,12 @@
   <x:dimension ref="A1:R34"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
-    <x:col min="1" max="2" width="19.453125" style="3" customWidth="1"/>
+    <x:col min="1" max="1" width="21.66796875" style="3" customWidth="1"/>
+    <x:col min="2" max="2" width="19.453125" style="3" customWidth="1"/>
     <x:col min="3" max="3" width="19.54296875" style="3" customWidth="1"/>
     <x:col min="4" max="4" width="50.7265625" style="3" customWidth="1"/>
     <x:col min="5" max="5" width="50.7265625" style="26" customWidth="1"/>
-    <x:col min="6" max="6" width="50.7265625" style="17" customWidth="1"/>
+    <x:col min="6" max="6" width="22.109375" style="17" customWidth="1"/>
     <x:col min="7" max="7" width="20.26953125" style="3" customWidth="1"/>
     <x:col min="8" max="8" width="30.54296875" style="3" customWidth="1"/>
     <x:col min="9" max="9" width="26.54296875" style="3" customWidth="1"/>
@@ -990,96 +1003,96 @@
   <x:sheetData>
     <x:row r="1" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
       <x:c r="D1" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E1" s="27"/>
       <x:c r="F1" s="18"/>
       <x:c r="G1" s="2"/>
       <x:c r="H1" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E2" s="27" t="s">
-        <x:v>9</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F2" s="18" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="I2" s="1"/>
     </x:row>
     <x:row r="3" spans="1:9" s="13" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="12" t="s">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="12" t="s">
-        <x:v>16</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C3" s="12" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D3" s="12" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E3" s="28" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F3" s="19" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E3" s="28" t="s">
+      <x:c r="G3" s="14" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H3" s="14" t="s">
         <x:v>20</x:v>
-      </x:c>
-      <x:c r="F3" s="19" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G3" s="14" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="H3" s="14" t="s">
-        <x:v>28</x:v>
       </x:c>
       <x:c r="I3" s="15"/>
     </x:row>
     <x:row r="4" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A4" s="4" t="s">
-        <x:v>25</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B4" s="4" t="s">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D4" s="4" t="s">
-        <x:v>23</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E4" s="29" t="s">
-        <x:v>11</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F4" s="20" t="s">
-        <x:v>24</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5" t="s">
-        <x:v>2</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="I4" s="16"/>
       <x:c r="J4" s="5"/>
@@ -1094,26 +1107,26 @@
     </x:row>
     <x:row r="5" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>15</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>29</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>10</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E5" s="30" t="s">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F5" s="21" t="s">
-        <x:v>30</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G5" s="5"/>
       <x:c r="H5" s="5" t="s">
-        <x:v>0</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="I5" s="5"/>
       <x:c r="J5" s="5"/>
@@ -1128,26 +1141,26 @@
     </x:row>
     <x:row r="6" spans="1:18" s="3" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A6" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B6" s="4" t="s">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="4" t="s">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D6" s="4" t="s">
-        <x:v>32</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E6" s="29" t="s">
-        <x:v>11</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F6" s="20" t="s">
-        <x:v>18</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G6" s="5"/>
       <x:c r="H6" s="5" t="s">
-        <x:v>1</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="I6" s="16"/>
       <x:c r="J6" s="5"/>
@@ -1161,14 +1174,24 @@
       <x:c r="R6" s="5"/>
     </x:row>
     <x:row r="7" spans="1:18" ht="15.75" customHeight="1">
-      <x:c r="A7" s="7"/>
-      <x:c r="B7" s="7"/>
-      <x:c r="C7" s="7"/>
+      <x:c r="A7" s="7" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="D7" s="7"/>
       <x:c r="E7" s="31"/>
-      <x:c r="F7" s="22"/>
+      <x:c r="F7" s="22" t="s">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="G7" s="5"/>
-      <x:c r="H7" s="5"/>
+      <x:c r="H7" s="5" t="s">
+        <x:v>35</x:v>
+      </x:c>
       <x:c r="I7" s="5"/>
       <x:c r="J7" s="5"/>
       <x:c r="K7" s="5"/>

</xml_diff>

<commit_message>
[Fix - Item + FieldObject Data] Id 수정 및 관련된 데이터 수정
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/FieldObject.xlsx
+++ b/JsonConverter/ExcelFiles/FieldObject.xlsx
@@ -21,106 +21,106 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <x:si>
+    <x:t>dropItem_GoldWellbeingCoin_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dropItem_wellbeingCoin_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>물약</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DPrefab/DropItem_TomatoJuice</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DPrefab/DropItem_CarrotSmoothy</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PrefabPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DropItem</x:t>
+  </x:si>
+  <x:si>
+    <x:t>황금 웰빙 코인</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_TomatoJuice_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dropItem_potion_1</x:t>
+  </x:si>
+  <x:si>
     <x:t>웰빙 코인</x:t>
   </x:si>
   <x:si>
-    <x:t>2DPrefab/DropItem_CarrotSmoothy</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DPrefab/DropItem_TomatoJuice</x:t>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>당근 스무디</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int[]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
   </x:si>
   <x:si>
     <x:t>(name)</x:t>
   </x:si>
   <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>당근 스무디</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int[]</x:t>
-  </x:si>
-  <x:si>
     <x:t>토마토 주스</x:t>
   </x:si>
   <x:si>
-    <x:t>PrefabPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DropItem</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>물약</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dropItem_potion_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_TomatoJuice_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dropItem_coin_1</x:t>
-  </x:si>
-  <x:si>
     <x:t>2DPrefab/DropItem_Potion</x:t>
   </x:si>
   <x:si>
     <x:t>dropItem_carrotSmoothy_1</x:t>
   </x:si>
   <x:si>
+    <x:t>Item_Potion_1</x:t>
+  </x:si>
+  <x:si>
     <x:t>DropCountRange</x:t>
   </x:si>
   <x:si>
+    <x:t>FieldObjectType</x:t>
+  </x:si>
+  <x:si>
+    <x:t>우선 프리팹으로 구현하자!</x:t>
+  </x:si>
+  <x:si>
     <x:t>DropItemDataId</x:t>
   </x:si>
   <x:si>
-    <x:t>우선 프리팹으로 구현하자!</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FieldObjectType</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Potion_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DPrefab/DropItem_Coin_2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DPrefab/DropItem_Coin_1</x:t>
-  </x:si>
-  <x:si>
     <x:t>dropItem_tomatoJuice_1</x:t>
   </x:si>
   <x:si>
     <x:t>Item_CarrotSmoothy_1</x:t>
   </x:si>
   <x:si>
-    <x:t>황금 웰빙 코인</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Coin_2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Coin_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dropItem_coin_2</x:t>
+    <x:t>2DPrefab/DropItem_WellbeingCoin_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_WellbeingCoin_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_GoldWellbeingCoin_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DPrefab/DropItem_GoldWellbeingCoin_1</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -971,21 +971,21 @@
   <x:dimension ref="A1:R34"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
-    <x:col min="1" max="1" width="23.77734375" style="3" customWidth="1"/>
+    <x:col min="1" max="1" width="27.47265625" style="3" bestFit="1" customWidth="1"/>
     <x:col min="2" max="2" width="19.453125" style="3" customWidth="1"/>
     <x:col min="3" max="3" width="19.54296875" style="3" customWidth="1"/>
     <x:col min="4" max="4" width="22.77734375" style="3" customWidth="1"/>
     <x:col min="5" max="5" width="20.22265625" style="24" customWidth="1"/>
-    <x:col min="6" max="6" width="22.109375" style="16" customWidth="1"/>
+    <x:col min="6" max="6" width="23.5546875" style="16" customWidth="1"/>
     <x:col min="7" max="7" width="20.26953125" style="3" customWidth="1"/>
-    <x:col min="8" max="8" width="30.54296875" style="3" customWidth="1"/>
+    <x:col min="8" max="8" width="34.4453125" style="3" customWidth="1"/>
     <x:col min="9" max="9" width="26.54296875" style="3" customWidth="1"/>
     <x:col min="10" max="16384" width="12.54296875" style="3"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -994,60 +994,60 @@
       <x:c r="F1" s="17"/>
       <x:c r="G1" s="2"/>
       <x:c r="H1" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E2" s="25" t="s">
-        <x:v>7</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F2" s="17" t="s">
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="I2" s="1"/>
     </x:row>
     <x:row r="3" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="11" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C3" s="11" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B3" s="11" t="s">
+      <x:c r="D3" s="11" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E3" s="26" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="C3" s="11" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D3" s="11" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E3" s="26" t="s">
-        <x:v>21</x:v>
-      </x:c>
       <x:c r="F3" s="18" t="s">
-        <x:v>22</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="G3" s="13" t="s">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H3" s="13" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="I3" s="14"/>
     </x:row>
@@ -1056,19 +1056,19 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B4" s="6" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C4" s="6" t="s">
-        <x:v>8</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D4" s="6"/>
       <x:c r="E4" s="28"/>
       <x:c r="F4" s="20" t="s">
-        <x:v>17</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5" t="s">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I4" s="5"/>
       <x:c r="J4" s="5"/>
@@ -1083,22 +1083,22 @@
     </x:row>
     <x:row r="5" spans="1:18" s="3" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>16</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>14</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="6"/>
       <x:c r="E5" s="28"/>
       <x:c r="F5" s="20" t="s">
-        <x:v>25</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G5" s="5"/>
       <x:c r="H5" s="5" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I5" s="5"/>
       <x:c r="J5" s="5"/>
@@ -1113,13 +1113,13 @@
     </x:row>
     <x:row r="6" spans="1:18" s="3" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A6" s="4" t="s">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B6" s="4" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="4" t="s">
-        <x:v>5</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D6" s="4"/>
       <x:c r="E6" s="27"/>
@@ -1128,7 +1128,7 @@
       </x:c>
       <x:c r="G6" s="5"/>
       <x:c r="H6" s="5" t="s">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I6" s="15"/>
       <x:c r="J6" s="5"/>
@@ -1143,22 +1143,22 @@
     </x:row>
     <x:row r="7" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>18</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C7" s="6" t="s">
-        <x:v>0</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D7" s="6"/>
       <x:c r="E7" s="28"/>
       <x:c r="F7" s="20" t="s">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G7" s="5"/>
       <x:c r="H7" s="5" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="I7" s="5"/>
       <x:c r="J7" s="5"/>
@@ -1173,22 +1173,22 @@
     </x:row>
     <x:row r="8" spans="1:18" s="3" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A8" s="6" t="s">
-        <x:v>33</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B8" s="6" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C8" s="6" t="s">
-        <x:v>30</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D8" s="6"/>
       <x:c r="E8" s="28"/>
       <x:c r="F8" s="20" t="s">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="G8" s="5"/>
       <x:c r="H8" s="5" t="s">
-        <x:v>26</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="I8" s="5"/>
       <x:c r="J8" s="5"/>

</xml_diff>